<commit_message>
RF03, RF04, RF05, RF06, requerimientos funcionales y user stories
</commit_message>
<xml_diff>
--- a/User stories.xlsx
+++ b/User stories.xlsx
@@ -5,18 +5,23 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALBERTO\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ceu365-my.sharepoint.com/personal/alberto_fernandezrodriguez_usp_ceu_es/Documents/UNI/Cuarto/Primer semestre/Ingeniería de sistemas de información/Ingeniería del software/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3289F115-A1A0-4817-B0DE-DA0D28E1E63C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{AFE3B115-B846-40BD-BAB0-234594C2838B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F76543C-2DCA-481D-A82C-DF1FACF3D239}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E227FCAF-17F8-4B51-A90D-51C2A08E46C6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{E227FCAF-17F8-4B51-A90D-51C2A08E46C6}"/>
   </bookViews>
   <sheets>
     <sheet name="US01 - RF01" sheetId="1" r:id="rId1"/>
     <sheet name="US02 - RF01" sheetId="2" r:id="rId2"/>
     <sheet name="US03 - RF02" sheetId="3" r:id="rId3"/>
     <sheet name="US04 - RF02" sheetId="4" r:id="rId4"/>
+    <sheet name="US05-RF03" sheetId="5" r:id="rId5"/>
+    <sheet name="US06-RF04" sheetId="6" r:id="rId6"/>
+    <sheet name="US07-RF05" sheetId="7" r:id="rId7"/>
+    <sheet name="US08-RF05" sheetId="8" r:id="rId8"/>
+    <sheet name="US09-RF06" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="62">
   <si>
     <r>
       <t xml:space="preserve">Como </t>
@@ -354,6 +359,547 @@
   </si>
   <si>
     <t>User Story 04 - RF02</t>
+  </si>
+  <si>
+    <t>User Story 05 - RF03</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Como usuario, quiero </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">crear un viaje </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">indicando origen/destino (texto + autocompletado), fecha/hora de salida, plazas y precio por plaza, para que el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>viaje quede publicado</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>El sistema requiere fecha y hora de salida para poder guardar el viaje.</t>
+  </si>
+  <si>
+    <t>El sistema requiere plazas y precio por plaza para poder guardar el viaje.</t>
+  </si>
+  <si>
+    <t>Al guardar con todos los campos válidos, el viaje queda creado/publicado y visible en el sistema.</t>
+  </si>
+  <si>
+    <t>El sistema permite introducir origen y destino como texto y ofrece sugerencias de autocompletado
+ al escribir.</t>
+  </si>
+  <si>
+    <t>El sistema permite introducir origen, destino y fecha como parámetros de búsqueda.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La búsqueda puede realizarse con </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uno o varios filtros</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Al ejecutar la búsqueda, el sistema muestra los </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>viajes que coinciden</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> con los parámetros indicados.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Si </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>no existen viajes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> que cumplan los criterios, el sistema muestra un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>mensaje informativo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+indicando que no hay resultados.</t>
+    </r>
+  </si>
+  <si>
+    <t>El sistema valida que la fecha introducida sea válida (no vacía, con formato correcto y no anterior a la fecha actual).</t>
+  </si>
+  <si>
+    <t>User Story 06 - RF04</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Como usuario, quiero </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">buscar viajes </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">indicando origen, destino y fecha, para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>encontrar los viajes que coinciden con mi búsqueda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Como usuario conductor, quiero </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">visualizar un listado con mis viajes </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>creados, para conocer su estado actual (publicado, pendiente, confirmado o cancelado).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El sistema muestra un listado denominado </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>“Mis viajes como conductor”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">En el listado aparecen </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>solo los viajes creados por el usuario autenticado</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> como conductor.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cada viaje muestra su </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>estado actual</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (publicado, pendiente, confirmado o cancelado).</t>
+    </r>
+  </si>
+  <si>
+    <t>El listado se actualiza automáticamente tras cada acción que modifique el estado del viaje.</t>
+  </si>
+  <si>
+    <t>User Story 07 - RF05</t>
+  </si>
+  <si>
+    <t>Como usuario pasajero, quiero visualizar un listado con mis reservas realizadas, para conocer su estado actual (pendiente, confirmado o cancelado).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El sistema muestra un listado denominado </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>“Mis reservas como pasajero”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">En el listado aparecen </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>solo las reservas realizadas por el usuario autenticado</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> como pasajero.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cada reserva muestra su </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>estado actual</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (pendiente, confirmado o cancelado).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El listado se </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>actualiza automáticamente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> cuando una reserva cambia de estado.</t>
+    </r>
+  </si>
+  <si>
+    <t>Como usuario pasajero, quiero reservar una plaza en un viaje disponible, para asegurar mi lugar como pasajero.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El sistema permite que un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>usuario pasajero</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> seleccione un viaje publicado y </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>reserve una plaza</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Al realizar la reserva, el sistema </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>reduce el número de plazas disponibles</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en ese viaje.</t>
+    </r>
+  </si>
+  <si>
+    <t>El sistema no permite realizar una reserva si no hay plazas disponibles (cupo completo).</t>
+  </si>
+  <si>
+    <t>El sistema no permite al mismo pasajero reservar dos veces el mismo viaje.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tras una reserva exitosa, el sistema </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>muestra confirmación</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y el viaje aparece en el listado
+ “Mis reservas como pasajero”.</t>
+    </r>
+  </si>
+  <si>
+    <t>User Story 09 - RF06</t>
+  </si>
+  <si>
+    <t>User Story 08 - RF05</t>
   </si>
 </sst>
 </file>
@@ -404,7 +950,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -464,12 +1010,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -500,6 +1077,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -508,6 +1100,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -525,6 +1132,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -862,7 +1473,7 @@
       <c r="D4" s="11"/>
     </row>
     <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="19" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -873,7 +1484,7 @@
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="15"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
@@ -882,7 +1493,7 @@
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="15"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="3" t="s">
         <v>3</v>
       </c>
@@ -891,7 +1502,7 @@
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="15"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="3" t="s">
         <v>4</v>
       </c>
@@ -900,7 +1511,7 @@
       </c>
     </row>
     <row r="9" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="16"/>
+      <c r="B9" s="21"/>
       <c r="C9" s="4" t="s">
         <v>5</v>
       </c>
@@ -993,7 +1604,7 @@
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="19" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1004,7 +1615,7 @@
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="15"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1013,7 +1624,7 @@
       </c>
     </row>
     <row r="7" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="15"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1108,7 +1719,7 @@
       <c r="D4" s="11"/>
     </row>
     <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="19" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1119,7 +1730,7 @@
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="15"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
         <v>18</v>
       </c>
@@ -1128,7 +1739,7 @@
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="15"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="3" t="s">
         <v>19</v>
       </c>
@@ -1137,7 +1748,7 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="15"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="4" t="s">
         <v>20</v>
       </c>
@@ -1230,10 +1841,10 @@
       <c r="D4" s="11"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="10">
@@ -1241,8 +1852,8 @@
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="15"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="20"/>
+      <c r="C6" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="10">
@@ -1250,8 +1861,8 @@
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="15"/>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="20"/>
+      <c r="C7" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="10">
@@ -1259,8 +1870,8 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="15"/>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="20"/>
+      <c r="C8" t="s">
         <v>25</v>
       </c>
       <c r="D8" s="10">
@@ -1330,4 +1941,632 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{296D9C4B-2505-4A55-8C1E-83A4FCFAE602}">
+  <dimension ref="B3:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="78.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="2:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="23"/>
+      <c r="C6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="23"/>
+      <c r="C7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="23"/>
+      <c r="C8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="15">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="7">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:B8"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D8">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{7F2ADDA7-67D5-431E-9B18-282F89DA72E4}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{7F2ADDA7-67D5-431E-9B18-282F89DA72E4}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D5:D8</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF831C71-0AA2-4595-8E27-E180FA8D8ADF}">
+  <dimension ref="B3:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="79.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="20"/>
+      <c r="C6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="20"/>
+      <c r="C7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B8" s="20"/>
+      <c r="C8" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="21"/>
+      <c r="C9" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="15">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="7">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:B9"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D9">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{9EC577B2-DFB1-45B9-AF3B-EA44007AC904}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{9EC577B2-DFB1-45B9-AF3B-EA44007AC904}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D5:D9</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A6E9D58-4463-4E07-AACF-E3E9083FC3D5}">
+  <dimension ref="B3:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="79.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="23"/>
+      <c r="C6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="23"/>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="23"/>
+      <c r="C8" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="15">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="7">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:B8"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D8">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{E22E35C2-51F7-4D1A-8015-BDA5983A5A8C}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{E22E35C2-51F7-4D1A-8015-BDA5983A5A8C}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D5:D8</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{065FFD8D-3A34-4138-8FFC-D60E521D1ECF}">
+  <dimension ref="B3:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="79.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="23"/>
+      <c r="C6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="23"/>
+      <c r="C7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="23"/>
+      <c r="C8" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="15">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="7">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:B8"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D8">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{C7E60796-F3ED-4580-B724-DBCFBA5222D6}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{C7E60796-F3ED-4580-B724-DBCFBA5222D6}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D5:D8</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7652FE5B-09C2-4A2D-80AB-B3085BA9E638}">
+  <dimension ref="B3:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="79.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="23"/>
+      <c r="C6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="23"/>
+      <c r="C7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="23"/>
+      <c r="C8" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="25"/>
+      <c r="C9" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="15">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="7">
+        <v>45958</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:B9"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D9">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{9509BB5D-4C86-4009-85F9-F3E268BD9BBE}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{9509BB5D-4C86-4009-85F9-F3E268BD9BBE}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D5:D9</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>